<commit_message>
fix(import): gabungkan baris orang yang sama bila salah satu baris tanpa tanggal lahir
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/buku2026-mini.xlsx
+++ b/tests/fixtures/buku2026-mini.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="42">
   <si>
     <t>NAMA</t>
   </si>
@@ -46,6 +46,18 @@
     <t>Anggota</t>
   </si>
   <si>
+    <t>DEWI MERGE TEST</t>
+  </si>
+  <si>
+    <t>Sekretaris</t>
+  </si>
+  <si>
+    <t>P</t>
+  </si>
+  <si>
+    <t>Jl. Merge Tetap</t>
+  </si>
+  <si>
     <t>KEDUDUKAN</t>
   </si>
   <si>
@@ -61,9 +73,6 @@
     <t>SITI KADAR UMUM</t>
   </si>
   <si>
-    <t>P</t>
-  </si>
-  <si>
     <t>v</t>
   </si>
   <si>
@@ -77,6 +86,24 @@
   </si>
   <si>
     <t>1988-03-20</t>
+  </si>
+  <si>
+    <t>SEKRETARIS</t>
+  </si>
+  <si>
+    <t>06 Februari 1976</t>
+  </si>
+  <si>
+    <t>RINA BEDA TGL</t>
+  </si>
+  <si>
+    <t>1980-01-01</t>
+  </si>
+  <si>
+    <t>Bendahara</t>
+  </si>
+  <si>
+    <t>1990-01-01</t>
   </si>
   <si>
     <t>2026-01-15</t>
@@ -455,10 +482,10 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:I14"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
-    <row r="9" spans="1:7">
+    <row r="9" spans="1:9">
       <c r="C9" t="s">
         <v>0</v>
       </c>
@@ -472,7 +499,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:7">
+    <row r="12" spans="1:9">
       <c r="C12" t="s">
         <v>4</v>
       </c>
@@ -486,9 +513,23 @@
         <v>7</v>
       </c>
     </row>
-    <row r="13" spans="1:7">
+    <row r="13" spans="1:9">
       <c r="D13" t="s">
         <v>8</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9">
+      <c r="C14" t="s">
+        <v>9</v>
+      </c>
+      <c r="D14" t="s">
+        <v>10</v>
+      </c>
+      <c r="E14" t="s">
+        <v>11</v>
+      </c>
+      <c r="I14" t="s">
+        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -503,7 +544,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:I14"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="9" spans="1:9">
@@ -511,13 +552,13 @@
         <v>0</v>
       </c>
       <c r="E9" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="F9" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="I9" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
     </row>
     <row r="12" spans="1:9">
@@ -528,7 +569,7 @@
         <v>6</v>
       </c>
       <c r="F12" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="I12" t="s">
         <v>7</v>
@@ -536,33 +577,75 @@
     </row>
     <row r="13" spans="1:9">
       <c r="D13" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="E13" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G13" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="I13" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
     </row>
     <row r="14" spans="1:9">
       <c r="D14" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E14" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F14" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="H14">
         <v>1</v>
       </c>
       <c r="I14" t="s">
-        <v>19</v>
+        <v>22</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9">
+      <c r="D15" t="s">
+        <v>9</v>
+      </c>
+      <c r="E15" t="s">
+        <v>11</v>
+      </c>
+      <c r="F15" t="s">
+        <v>23</v>
+      </c>
+      <c r="I15" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9">
+      <c r="D16" t="s">
+        <v>25</v>
+      </c>
+      <c r="E16" t="s">
+        <v>11</v>
+      </c>
+      <c r="F16" t="s">
+        <v>8</v>
+      </c>
+      <c r="I16" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9">
+      <c r="D17" t="s">
+        <v>25</v>
+      </c>
+      <c r="E17" t="s">
+        <v>11</v>
+      </c>
+      <c r="F17" t="s">
+        <v>27</v>
+      </c>
+      <c r="I17" t="s">
+        <v>28</v>
       </c>
     </row>
   </sheetData>
@@ -585,19 +668,19 @@
         <v>1</v>
       </c>
       <c r="C9" t="s">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="D9" t="s">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="E9" t="s">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="F9" t="s">
-        <v>23</v>
+        <v>32</v>
       </c>
       <c r="G9" t="s">
-        <v>24</v>
+        <v>33</v>
       </c>
     </row>
     <row r="11" spans="1:14">
@@ -605,28 +688,28 @@
         <v>2</v>
       </c>
       <c r="C11" t="s">
-        <v>25</v>
+        <v>34</v>
       </c>
       <c r="E11" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="F11" t="s">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="G11" t="s">
-        <v>28</v>
+        <v>37</v>
       </c>
       <c r="K11" t="s">
-        <v>29</v>
+        <v>38</v>
       </c>
       <c r="L11" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="M11" t="s">
-        <v>31</v>
+        <v>40</v>
       </c>
       <c r="N11" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
     </row>
   </sheetData>

</xml_diff>